<commit_message>
Improve V2 retrieval accuracy and resilience
</commit_message>
<xml_diff>
--- a/knowledge-source/功能知识库.xlsx
+++ b/knowledge-source/功能知识库.xlsx
@@ -669,12 +669,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>创建环境</t>
+          <t>创建环境,创建浏览器</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>create profile</t>
+          <t>create profile,create browser</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -4982,12 +4982,12 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>操作日志</t>
+          <t>操作日志,查询操作记录,查询操作者,谁修改了环境,查看环境修改记录,在哪里看环境操作者,查询环境配置变更记录</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>operation log</t>
+          <t>operation log, query operation records, query operator, who modified the profile, view the profile modification records, where to see the profile operator, query the profile configuration change records</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -6206,12 +6206,12 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>浏览器内核</t>
+          <t>浏览器内核,修改浏览器内核,修改内核版本,编辑环境内核版本</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>browser kernel</t>
+          <t>browser kernel, modify browser kernel, modify kernel version, edit profile kernel version</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">

</xml_diff>